<commit_message>
Updated Documentation For Sprint
1. Updated Product Backlog
2. Updated WireFrames
3. Updated UseCaseScenarios
4. Updated UseCaseDiagram
</commit_message>
<xml_diff>
--- a/documentation/Product Backlog.xlsx
+++ b/documentation/Product Backlog.xlsx
@@ -1,31 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29518"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jcorley\OneDrive - University of West Georgia\Teaching\Software Engineering I\SE1-Fall 25\Projects\Project 1\Pirate Ship Inventory System Design Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53D7C448-58BF-4D33-BF0A-49D0CABEBD7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{25BF5A00-7FFF-4C48-880E-30510124E0DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="13845" windowHeight="22620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
+  <si>
+    <t>Priority</t>
+  </si>
   <si>
     <t>As a…</t>
   </si>
@@ -36,9 +50,6 @@
     <t>So that…</t>
   </si>
   <si>
-    <t>Priority</t>
-  </si>
-  <si>
     <t>Crewmate</t>
   </si>
   <si>
@@ -51,9 +62,18 @@
     <t>Quartermaster</t>
   </si>
   <si>
+    <t>to review stock changes</t>
+  </si>
+  <si>
     <t>I can ensure all stock is being managed properly</t>
   </si>
   <si>
+    <t>to review the whole inventory</t>
+  </si>
+  <si>
+    <t>I can determine what is in the inventory</t>
+  </si>
+  <si>
     <t>Cook</t>
   </si>
   <si>
@@ -69,6 +89,9 @@
     <t>I can cook it</t>
   </si>
   <si>
+    <t>Officer</t>
+  </si>
+  <si>
     <t>to see what munitions are available</t>
   </si>
   <si>
@@ -81,9 +104,6 @@
     <t>I can use it to engage in combat</t>
   </si>
   <si>
-    <t>Officer</t>
-  </si>
-  <si>
     <t>to report damage</t>
   </si>
   <si>
@@ -115,16 +135,13 @@
   </si>
   <si>
     <t>I can control who has access to the system and how they can use the system</t>
-  </si>
-  <si>
-    <t>to review stock changes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -477,8 +494,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
@@ -486,21 +503,21 @@
     <col min="4" max="4" width="69.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -514,7 +531,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -522,18 +539,18 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="3">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>10</v>
@@ -542,82 +559,82 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4">
       <c r="A5" s="3">
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="3">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
-        <v>3</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="4">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="D7" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="4">
+        <v>3</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="5">
-        <v>4</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D8" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" s="5">
         <v>4</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="5">
         <v>4</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>24</v>
@@ -626,32 +643,46 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4">
       <c r="A11" s="5">
         <v>4</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="6">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="5">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="6">
         <v>5</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>29</v>
+      <c r="B13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>